<commit_message>
Income & Expense pages
</commit_message>
<xml_diff>
--- a/backend/expenses_details.xlsx
+++ b/backend/expenses_details.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,18 +413,51 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Gas</v>
+        <v>Rent</v>
       </c>
       <c r="B2">
-        <v>500</v>
+        <v>850</v>
       </c>
       <c r="C2" s="1">
+        <v>46104.791666666664</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="B3">
+        <v>120</v>
+      </c>
+      <c r="C3" s="1">
+        <v>46101.791666666664</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Tuition</v>
+      </c>
+      <c r="B4">
+        <v>7500</v>
+      </c>
+      <c r="C4" s="1">
         <v>46100.791666666664</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Nike</v>
+      </c>
+      <c r="B5">
+        <v>76</v>
+      </c>
+      <c r="C5" s="1">
+        <v>46092.791666666664</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dark theme, Charts` filter, chat-bot
</commit_message>
<xml_diff>
--- a/backend/expenses_details.xlsx
+++ b/backend/expenses_details.xlsx
@@ -413,46 +413,46 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Rent</v>
+        <v>Gas</v>
       </c>
       <c r="B2">
-        <v>850</v>
+        <v>100</v>
       </c>
       <c r="C2" s="1">
-        <v>46104.791666666664</v>
+        <v>46099.791666666664</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Groceries</v>
+        <v>Rent</v>
       </c>
       <c r="B3">
-        <v>120</v>
+        <v>1000</v>
       </c>
       <c r="C3" s="1">
-        <v>46101.791666666664</v>
+        <v>46081.75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Tuition</v>
+        <v>Grad School Application Fee</v>
       </c>
       <c r="B4">
-        <v>7500</v>
+        <v>1750</v>
       </c>
       <c r="C4" s="1">
-        <v>46100.791666666664</v>
+        <v>46005.75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nike</v>
+        <v>Gift for Friend`s Birthday</v>
       </c>
       <c r="B5">
-        <v>76</v>
+        <v>350</v>
       </c>
       <c r="C5" s="1">
-        <v>46092.791666666664</v>
+        <v>45993.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>